<commit_message>
Fix date shown on jury sheet
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/jury/Jury-A4.xlsx
+++ b/owlcms/src/main/resources/templates/jury/Jury-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\jury\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\jury\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C49C247-EBD9-40FC-BA69-EBE2BEDFF35D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9CBE2A3-1B88-4A4A-AC75-B4B18A798804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41490" yWindow="-3705" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jury" sheetId="1" r:id="rId1"/>
@@ -74,9 +74,6 @@
     <t>${competition.competitionSite}</t>
   </si>
   <si>
-    <t>${competition.competitionDate}</t>
-  </si>
-  <si>
     <t>${session.referee1}</t>
   </si>
   <si>
@@ -150,6 +147,9 @@
   </si>
   <si>
     <t>${t.get("Jury.Signature")}</t>
+  </si>
+  <si>
+    <t>${session.competitionTimeAsExcelDate}</t>
   </si>
 </sst>
 </file>
@@ -601,15 +601,7 @@
     <cellStyle name="Titre 1 1 1 1 1" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
     <cellStyle name="Titre de la feuille" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="34"/>
-          <bgColor indexed="13"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1144,7 +1136,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B1" s="40"/>
       <c r="C1" s="40"/>
@@ -1160,7 +1152,7 @@
     </row>
     <row r="2" spans="1:12" ht="27.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="46" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="46"/>
       <c r="C2" s="2" t="s">
@@ -1172,16 +1164,16 @@
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
       <c r="I2" s="27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J2" s="36" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K2" s="25"/>
     </row>
     <row r="3" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="46" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="46"/>
       <c r="C3" s="47" t="s">
@@ -1191,23 +1183,23 @@
       <c r="E3" s="47"/>
       <c r="F3" s="47"/>
       <c r="G3" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H3" s="30" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="I3" s="27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J3" s="36" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3" s="25"/>
     </row>
     <row r="4" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="41" t="s">
         <v>1</v>
@@ -1218,10 +1210,10 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J4" s="36" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K4" s="25"/>
     </row>
@@ -1232,12 +1224,12 @@
       <c r="C6" s="7"/>
       <c r="D6" s="8"/>
       <c r="F6" s="42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G6" s="43"/>
       <c r="H6" s="44"/>
       <c r="I6" s="43" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" s="43"/>
       <c r="K6" s="45"/>
@@ -1247,14 +1239,14 @@
         <v>0</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="49"/>
       <c r="D7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>17</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>18</v>
       </c>
       <c r="F7" s="9">
         <v>1</v>
@@ -1277,22 +1269,22 @@
     </row>
     <row r="8" spans="1:12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="51"/>
       <c r="D9" s="29" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="33" t="s">
         <v>24</v>
-      </c>
-      <c r="E9" s="33" t="s">
-        <v>25</v>
       </c>
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
@@ -1303,7 +1295,7 @@
     </row>
     <row r="10" spans="1:12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -1319,18 +1311,18 @@
     </row>
     <row r="12" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="39" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="39"/>
       <c r="C12" s="16"/>
       <c r="D12" s="17"/>
       <c r="E12" s="18"/>
       <c r="F12" s="20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G12" s="19"/>
       <c r="H12" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I12" s="37"/>
       <c r="J12" s="38"/>
@@ -1564,21 +1556,16 @@
     <mergeCell ref="B9:C9"/>
   </mergeCells>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11 C12 J12">
-    <cfRule type="expression" dxfId="2" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="8" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D9:D10">
-    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
-      <formula>AND((#REF!),#REF!,#REF!)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9:E10">
+  <conditionalFormatting sqref="D9:E10">
     <cfRule type="expression" dxfId="0" priority="3" stopIfTrue="1">
       <formula>AND((#REF!),#REF!,#REF!)</formula>
     </cfRule>

</xml_diff>